<commit_message>
Updated events for credit note spelling
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst_ALT/ActivityData/BillType.xlsx
+++ b/src/test/resources/TestDriver/Hearst_ALT/ActivityData/BillType.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b68cc7b829e61597/Desktop/Hearst_Project/Sandbox/RefData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst_CDB\ActivityData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{963440CE-1DF8-4E1E-B543-310A9AF8F5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FF4DB18-2530-46F6-B8A4-7185A3F0F4CA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411B9014-8035-4E69-9822-51E8EDF52D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Billing_Type</t>
   </si>
@@ -46,12 +46,15 @@
   <si>
     <t>CREDITNOTE</t>
   </si>
+  <si>
+    <t>CREDIT NOTE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -60,6 +63,13 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -87,9 +97,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -105,10 +116,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -309,7 +316,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1194FE4C-FBC1-4D63-8FD6-C5A14E8D6200}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
@@ -326,8 +333,13 @@
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>